<commit_message>
New tests + fixes (#4)
* New test test_search_only_city

* New test test_dropdown_click

* proof_location fix

* dropdown_click fix

* dropdown_click fix2

* cancel_registration_window add

* add_destination fix
proof_hotel add

* add_destination fix

* add_destination_by_dropdown add
test_dropdown_click fix
</commit_message>
<xml_diff>
--- a/testcases/testcases.xlsx
+++ b/testcases/testcases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47A3A0A-5DE2-441D-A10A-09DEF9D06CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D90FC8E-75FF-4FE5-9AE2-E2360473BFB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="125">
   <si>
     <t>№</t>
   </si>
@@ -418,6 +418,31 @@
   </si>
   <si>
     <t>pytest -k test_search_only_city -sv</t>
+  </si>
+  <si>
+    <t>TC-SRCH-10</t>
+  </si>
+  <si>
+    <t>Recent searches</t>
+  </si>
+  <si>
+    <t>1. In the "Where to?" field, enter "Belgrade".
+2. Click "Search"
+3. In the "Where to?" field, enter "Moscow".
+4. Click "Search"
+5. In the "Where to?" field, enter "Hamburg".
+6. Click "Search"
+7. Click "Where to go" field
+8. Choose "Belgrade" from the dropdown list</t>
+  </si>
+  <si>
+    <t>The search results page opens, displaying hotels in Belgrade.</t>
+  </si>
+  <si>
+    <t>test_dropdown_click</t>
+  </si>
+  <si>
+    <t>pytest -k test_dropdown_click -sv</t>
   </si>
 </sst>
 </file>
@@ -453,7 +478,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -463,6 +488,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -505,7 +536,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -539,6 +570,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -820,7 +870,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -859,47 +909,56 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
+    <row r="2" spans="1:8" s="16" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="58" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
+    <row r="3" spans="1:8" s="16" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="14" t="s">
         <v>12</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -1019,6 +1078,23 @@
       </c>
       <c r="E10" s="5" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="116" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>